<commit_message>
Cambiando columnas de fecha con formato dia/mes/año
</commit_message>
<xml_diff>
--- a/reporte_trading/reporte_trading.xlsx
+++ b/reporte_trading/reporte_trading.xlsx
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,7 +55,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,8 +421,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -436,50 +454,65 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>trades_ganados</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>trades_perdidos</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>trades_empate</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>total_invertido</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>total_vendido</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>pnl_total</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>trade_mas_ganador</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>trade_mas_perdedor</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>roi_total</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>roi_promedio</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>mejor_trade</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>peor_trade</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>winrate</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>roi_total</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>cantidad_abierta</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>costo_abierto</t>
         </is>
@@ -495,19 +528,19 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
         <v>1500</v>
       </c>
-      <c r="D2" t="n">
+      <c r="G2" t="n">
         <v>1600</v>
-      </c>
-      <c r="E2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F2" t="n">
-        <v>6.666666666666667</v>
-      </c>
-      <c r="G2" t="n">
-        <v>100</v>
       </c>
       <c r="H2" t="n">
         <v>100</v>
@@ -516,12 +549,21 @@
         <v>100</v>
       </c>
       <c r="J2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K2" t="n">
         <v>6.666666666666667</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
       <c r="L2" t="n">
+        <v>6.666666666666667</v>
+      </c>
+      <c r="M2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -535,19 +577,19 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
         <v>1500</v>
       </c>
-      <c r="D3" t="n">
+      <c r="G3" t="n">
         <v>1600</v>
-      </c>
-      <c r="E3" t="n">
-        <v>100</v>
-      </c>
-      <c r="F3" t="n">
-        <v>6.666666666666667</v>
-      </c>
-      <c r="G3" t="n">
-        <v>100</v>
       </c>
       <c r="H3" t="n">
         <v>100</v>
@@ -556,12 +598,21 @@
         <v>100</v>
       </c>
       <c r="J3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K3" t="n">
         <v>6.666666666666667</v>
       </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
       <c r="L3" t="n">
+        <v>6.666666666666667</v>
+      </c>
+      <c r="M3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -575,33 +626,42 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
         <v>120</v>
       </c>
-      <c r="D4" t="n">
+      <c r="G4" t="n">
         <v>150</v>
-      </c>
-      <c r="E4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" t="n">
-        <v>25</v>
-      </c>
-      <c r="G4" t="n">
-        <v>30</v>
       </c>
       <c r="H4" t="n">
         <v>30</v>
       </c>
       <c r="I4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J4" t="n">
+        <v>30</v>
+      </c>
+      <c r="K4" t="n">
+        <v>25</v>
+      </c>
+      <c r="L4" t="n">
+        <v>25</v>
+      </c>
+      <c r="M4" t="n">
         <v>100</v>
       </c>
-      <c r="J4" t="n">
-        <v>25</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -615,33 +675,42 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
         <v>200</v>
       </c>
-      <c r="D5" t="n">
+      <c r="G5" t="n">
         <v>220</v>
-      </c>
-      <c r="E5" t="n">
-        <v>20.00000000000003</v>
-      </c>
-      <c r="F5" t="n">
-        <v>10.00000000000001</v>
-      </c>
-      <c r="G5" t="n">
-        <v>20.00000000000003</v>
       </c>
       <c r="H5" t="n">
         <v>20.00000000000003</v>
       </c>
       <c r="I5" t="n">
+        <v>20.00000000000003</v>
+      </c>
+      <c r="J5" t="n">
+        <v>20.00000000000003</v>
+      </c>
+      <c r="K5" t="n">
+        <v>10.00000000000001</v>
+      </c>
+      <c r="L5" t="n">
+        <v>10.00000000000001</v>
+      </c>
+      <c r="M5" t="n">
         <v>100</v>
       </c>
-      <c r="J5" t="n">
-        <v>10.00000000000001</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -655,33 +724,42 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>500</v>
       </c>
-      <c r="D6" t="n">
+      <c r="G6" t="n">
         <v>520</v>
-      </c>
-      <c r="E6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" t="n">
-        <v>20</v>
       </c>
       <c r="H6" t="n">
         <v>20</v>
       </c>
       <c r="I6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" t="n">
         <v>100</v>
       </c>
-      <c r="J6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -695,33 +773,42 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
         <v>30</v>
       </c>
-      <c r="D7" t="n">
+      <c r="G7" t="n">
         <v>36</v>
-      </c>
-      <c r="E7" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G7" t="n">
-        <v>6</v>
       </c>
       <c r="H7" t="n">
         <v>6</v>
       </c>
       <c r="I7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" t="n">
+        <v>20</v>
+      </c>
+      <c r="M7" t="n">
         <v>100</v>
       </c>
-      <c r="J7" t="n">
-        <v>20</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -735,33 +822,42 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
         <v>50</v>
       </c>
-      <c r="D8" t="n">
+      <c r="G8" t="n">
         <v>45</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-10</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-5</v>
       </c>
       <c r="H8" t="n">
         <v>-5</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="J8" t="n">
+        <v>-5</v>
+      </c>
+      <c r="K8" t="n">
         <v>-10</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
       <c r="L8" t="n">
+        <v>-10</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -776,8 +872,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -785,47 +895,57 @@
           <t>Moneda</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Fecha compra inicial</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Fecha venta</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Precio compra promedio</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Cantidad vendida</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Precio compra</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>Precio venta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Costo USDT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Venta USDT</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PnL USDT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ROI %</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
@@ -837,31 +957,41 @@
           <t>ADA</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>45361.39583333334</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>45366.59722222222</v>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>10/03/24</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>15/03/24</t>
+        </is>
       </c>
       <c r="D2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E2" t="n">
         <v>100</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G2" t="n">
         <v>1.5</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>120</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>150</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>30</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>25</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
@@ -873,31 +1003,41 @@
           <t>AXS</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>45332.75</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>45337.77083333334</v>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>10/02/24</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>15/02/24</t>
+        </is>
       </c>
       <c r="D3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E3" t="n">
         <v>20</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G3" t="n">
         <v>1.8</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>30</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>36</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>6</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>20</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
@@ -909,31 +1049,41 @@
           <t>BNB</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>45383.45833333334</v>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>45385.45833333334</v>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>01/04/24</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>03/04/24</t>
+        </is>
       </c>
       <c r="D4" t="n">
+        <v>300</v>
+      </c>
+      <c r="E4" t="n">
         <v>5</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G4" t="n">
         <v>320</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>1500</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>1600</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
         <v>100</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>6.666666666666667</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
@@ -945,31 +1095,41 @@
           <t>BTC</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>45301.39583333334</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>45306.59722222222</v>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>10/01/24</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>15/01/24</t>
+        </is>
       </c>
       <c r="D5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.01</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G5" t="n">
         <v>52000</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>500</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>520</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
         <v>20</v>
       </c>
-      <c r="I5" t="n">
+      <c r="K5" t="n">
         <v>4</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
@@ -981,31 +1141,41 @@
           <t>DOT</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
-        <v>45292.41666666666</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>45296.5</v>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>01/01/24</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>05/01/24</t>
+        </is>
       </c>
       <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
         <v>100</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
         <v>2.2</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>200</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>220</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>20.00000000000003</v>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>10.00000000000001</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
@@ -1017,31 +1187,41 @@
           <t>ETH</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
-        <v>45352.41666666666</v>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>45356.5</v>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>01/03/24</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>05/03/24</t>
+        </is>
       </c>
       <c r="D7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.5</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G7" t="n">
         <v>3200</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>1500</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>1600</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
         <v>100</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>6.666666666666667</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
@@ -1053,31 +1233,41 @@
           <t>UNI</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
-        <v>45323.45833333334</v>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>45325.45833333334</v>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>01/02/24</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>03/02/24</t>
+        </is>
       </c>
       <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
         <v>10</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
         <v>4.5</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>50</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>45</v>
       </c>
-      <c r="H8" t="n">
+      <c r="J8" t="n">
         <v>-5</v>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>-10</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Pérdida</t>
         </is>
@@ -1109,6 +1299,26 @@
   </sheetPr>
   <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1171,7 +1381,7 @@
           <t>Estado</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
@@ -1205,15 +1415,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>24-01-01 10:00:00</t>
+          <t>24-03-10 09:30:00</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1001</v>
+        <v>1011</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOTUSDT</t>
+          <t>ADAUSDT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1231,25 +1441,25 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>100DOT</t>
+          <t>100ADA</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>24-01-01 10:00:00</t>
+          <t>24-03-10 09:30:00</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>100DOT</t>
+          <t>100ADA</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>200USDT</t>
+          <t>120USDT</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1258,20 +1468,20 @@
         </is>
       </c>
       <c r="M2" s="1" t="n">
-        <v>45292.41666666666</v>
+        <v>45361.39583333334</v>
       </c>
       <c r="N2" t="n">
         <v>100</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="P2" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DOT</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -1283,15 +1493,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>24-01-05 12:00:00</t>
+          <t>24-03-15 14:20:00</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1002</v>
+        <v>1012</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DOTUSDT</t>
+          <t>ADAUSDT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1309,25 +1519,25 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>100DOT</t>
+          <t>100ADA</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>24-01-05 12:00:00</t>
+          <t>24-03-15 14:20:00</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>100DOT</t>
+          <t>100ADA</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>220USDT</t>
+          <t>150USDT</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1336,20 +1546,20 @@
         </is>
       </c>
       <c r="M3" s="1" t="n">
-        <v>45296.5</v>
+        <v>45366.59722222222</v>
       </c>
       <c r="N3" t="n">
         <v>100</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="P3" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>DOT</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1361,15 +1571,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>24-01-10 09:30:00</t>
+          <t>24-02-10 18:00:00</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BTCUSDT</t>
+          <t>AXSUSDT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1387,25 +1597,25 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.01BTC</t>
+          <t>20AXS</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>24-01-10 09:30:00</t>
+          <t>24-02-10 18:00:00</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.01BTC</t>
+          <t>20AXS</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>50000</v>
+        <v>1.5</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>500USDT</t>
+          <t>30USDT</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1414,20 +1624,20 @@
         </is>
       </c>
       <c r="M4" s="1" t="n">
-        <v>45301.39583333334</v>
+        <v>45332.75</v>
       </c>
       <c r="N4" t="n">
-        <v>0.01</v>
+        <v>20</v>
       </c>
       <c r="O4" t="n">
-        <v>50000</v>
+        <v>1.5</v>
       </c>
       <c r="P4" t="n">
-        <v>500</v>
+        <v>30</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -1439,15 +1649,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>24-01-15 14:20:00</t>
+          <t>24-02-15 18:30:00</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BTCUSDT</t>
+          <t>AXSUSDT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1465,25 +1675,25 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.01BTC</t>
+          <t>20AXS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>24-01-15 14:20:00</t>
+          <t>24-02-15 18:30:00</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.01BTC</t>
+          <t>20AXS</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>52000</v>
+        <v>1.8</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>520USDT</t>
+          <t>36USDT</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1492,20 +1702,20 @@
         </is>
       </c>
       <c r="M5" s="1" t="n">
-        <v>45306.59722222222</v>
+        <v>45337.77083333334</v>
       </c>
       <c r="N5" t="n">
-        <v>0.01</v>
+        <v>20</v>
       </c>
       <c r="O5" t="n">
-        <v>52000</v>
+        <v>1.8</v>
       </c>
       <c r="P5" t="n">
-        <v>520</v>
+        <v>36</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1517,15 +1727,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>24-02-01 11:00:00</t>
+          <t>24-04-01 11:00:00</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1005</v>
+        <v>1013</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>UNIUSDT</t>
+          <t>BNBUSDT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1543,47 +1753,47 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10UNI</t>
+          <t>5BNB</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>24-02-01 11:00:00</t>
+          <t>24-04-01 11:00:00</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>10UNI</t>
+          <t>5BNB</t>
         </is>
       </c>
       <c r="J6" t="n">
+        <v>300</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1500USDT</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="n">
+        <v>45383.45833333334</v>
+      </c>
+      <c r="N6" t="n">
         <v>5</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>50USDT</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>FILLED</t>
-        </is>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>45323.45833333334</v>
-      </c>
-      <c r="N6" t="n">
-        <v>10</v>
-      </c>
       <c r="O6" t="n">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="P6" t="n">
-        <v>50</v>
+        <v>1500</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>UNI</t>
+          <t>BNB</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1595,15 +1805,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>24-02-03 11:00:00</t>
+          <t>24-04-03 11:00:00</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1006</v>
+        <v>1014</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>UNIUSDT</t>
+          <t>BNBUSDT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1621,25 +1831,25 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10UNI</t>
+          <t>5BNB</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>24-02-03 11:00:00</t>
+          <t>24-04-03 11:00:00</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>10UNI</t>
+          <t>5BNB</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>4.5</v>
+        <v>320</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>45USDT</t>
+          <t>1600USDT</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1648,20 +1858,20 @@
         </is>
       </c>
       <c r="M7" s="1" t="n">
-        <v>45325.45833333334</v>
+        <v>45385.45833333334</v>
       </c>
       <c r="N7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O7" t="n">
-        <v>4.5</v>
+        <v>320</v>
       </c>
       <c r="P7" t="n">
-        <v>45</v>
+        <v>1600</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>UNI</t>
+          <t>BNB</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1673,15 +1883,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24-02-10 18:00:00</t>
+          <t>24-01-10 09:30:00</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AXSUSDT</t>
+          <t>BTCUSDT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1699,25 +1909,25 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>20AXS</t>
+          <t>0.01BTC</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>24-02-10 18:00:00</t>
+          <t>24-01-10 09:30:00</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>20AXS</t>
+          <t>0.01BTC</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1.5</v>
+        <v>50000</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>30USDT</t>
+          <t>500USDT</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1726,20 +1936,20 @@
         </is>
       </c>
       <c r="M8" s="1" t="n">
-        <v>45332.75</v>
+        <v>45301.39583333334</v>
       </c>
       <c r="N8" t="n">
-        <v>20</v>
+        <v>0.01</v>
       </c>
       <c r="O8" t="n">
-        <v>1.5</v>
+        <v>50000</v>
       </c>
       <c r="P8" t="n">
-        <v>30</v>
+        <v>500</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1751,15 +1961,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>24-02-15 18:30:00</t>
+          <t>24-01-15 14:20:00</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AXSUSDT</t>
+          <t>BTCUSDT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1777,25 +1987,25 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>20AXS</t>
+          <t>0.01BTC</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>24-02-15 18:30:00</t>
+          <t>24-01-15 14:20:00</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20AXS</t>
+          <t>0.01BTC</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1.8</v>
+        <v>52000</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>36USDT</t>
+          <t>520USDT</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1804,20 +2014,20 @@
         </is>
       </c>
       <c r="M9" s="1" t="n">
-        <v>45337.77083333334</v>
+        <v>45306.59722222222</v>
       </c>
       <c r="N9" t="n">
-        <v>20</v>
+        <v>0.01</v>
       </c>
       <c r="O9" t="n">
-        <v>1.8</v>
+        <v>52000</v>
       </c>
       <c r="P9" t="n">
-        <v>36</v>
+        <v>520</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1829,15 +2039,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>24-03-01 10:00:00</t>
+          <t>24-01-01 10:00:00</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1009</v>
+        <v>1001</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ETHUSDT</t>
+          <t>DOTUSDT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1855,25 +2065,25 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.5ETH</t>
+          <t>100DOT</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>24-03-01 10:00:00</t>
+          <t>24-01-01 10:00:00</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0.5ETH</t>
+          <t>100DOT</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3000</v>
+        <v>2</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1500USDT</t>
+          <t>200USDT</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1882,20 +2092,20 @@
         </is>
       </c>
       <c r="M10" s="1" t="n">
-        <v>45352.41666666666</v>
+        <v>45292.41666666666</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="O10" t="n">
-        <v>3000</v>
+        <v>2</v>
       </c>
       <c r="P10" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1907,15 +2117,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>24-03-05 12:00:00</t>
+          <t>24-01-05 12:00:00</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1010</v>
+        <v>1002</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ETHUSDT</t>
+          <t>DOTUSDT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1933,25 +2143,25 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.5ETH</t>
+          <t>100DOT</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>24-03-05 12:00:00</t>
+          <t>24-01-05 12:00:00</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.5ETH</t>
+          <t>100DOT</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3200</v>
+        <v>2.2</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1600USDT</t>
+          <t>220USDT</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1960,20 +2170,20 @@
         </is>
       </c>
       <c r="M11" s="1" t="n">
-        <v>45356.5</v>
+        <v>45296.5</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="O11" t="n">
-        <v>3200</v>
+        <v>2.2</v>
       </c>
       <c r="P11" t="n">
-        <v>1600</v>
+        <v>220</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1985,15 +2195,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>24-03-10 09:30:00</t>
+          <t>24-03-01 10:00:00</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ADAUSDT</t>
+          <t>ETHUSDT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2011,25 +2221,25 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>100ADA</t>
+          <t>0.5ETH</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>24-03-10 09:30:00</t>
+          <t>24-03-01 10:00:00</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>100ADA</t>
+          <t>0.5ETH</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>1.2</v>
+        <v>3000</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>120USDT</t>
+          <t>1500USDT</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2038,20 +2248,20 @@
         </is>
       </c>
       <c r="M12" s="1" t="n">
-        <v>45361.39583333334</v>
+        <v>45352.41666666666</v>
       </c>
       <c r="N12" t="n">
-        <v>100</v>
+        <v>0.5</v>
       </c>
       <c r="O12" t="n">
-        <v>1.2</v>
+        <v>3000</v>
       </c>
       <c r="P12" t="n">
-        <v>120</v>
+        <v>1500</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -2063,15 +2273,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>24-03-15 14:20:00</t>
+          <t>24-03-05 12:00:00</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ADAUSDT</t>
+          <t>ETHUSDT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2089,25 +2299,25 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>100ADA</t>
+          <t>0.5ETH</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>24-03-15 14:20:00</t>
+          <t>24-03-05 12:00:00</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>100ADA</t>
+          <t>0.5ETH</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>1.5</v>
+        <v>3200</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>150USDT</t>
+          <t>1600USDT</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2116,20 +2326,20 @@
         </is>
       </c>
       <c r="M13" s="1" t="n">
-        <v>45366.59722222222</v>
+        <v>45356.5</v>
       </c>
       <c r="N13" t="n">
-        <v>100</v>
+        <v>0.5</v>
       </c>
       <c r="O13" t="n">
-        <v>1.5</v>
+        <v>3200</v>
       </c>
       <c r="P13" t="n">
-        <v>150</v>
+        <v>1600</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -2141,15 +2351,15 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>24-04-01 11:00:00</t>
+          <t>24-02-01 11:00:00</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1013</v>
+        <v>1005</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BNBUSDT</t>
+          <t>UNIUSDT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2167,25 +2377,25 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5BNB</t>
+          <t>10UNI</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>24-04-01 11:00:00</t>
+          <t>24-02-01 11:00:00</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>5BNB</t>
+          <t>10UNI</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>300</v>
+        <v>5</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1500USDT</t>
+          <t>50USDT</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2194,20 +2404,20 @@
         </is>
       </c>
       <c r="M14" s="1" t="n">
-        <v>45383.45833333334</v>
+        <v>45323.45833333334</v>
       </c>
       <c r="N14" t="n">
+        <v>10</v>
+      </c>
+      <c r="O14" t="n">
         <v>5</v>
       </c>
-      <c r="O14" t="n">
-        <v>300</v>
-      </c>
       <c r="P14" t="n">
-        <v>1500</v>
+        <v>50</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>BNB</t>
+          <t>UNI</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -2219,15 +2429,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>24-04-03 11:00:00</t>
+          <t>24-02-03 11:00:00</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1014</v>
+        <v>1006</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BNBUSDT</t>
+          <t>UNIUSDT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2245,25 +2455,25 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5BNB</t>
+          <t>10UNI</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>24-04-03 11:00:00</t>
+          <t>24-02-03 11:00:00</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>5BNB</t>
+          <t>10UNI</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>320</v>
+        <v>4.5</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1600USDT</t>
+          <t>45USDT</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2272,20 +2482,20 @@
         </is>
       </c>
       <c r="M15" s="1" t="n">
-        <v>45385.45833333334</v>
+        <v>45325.45833333334</v>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O15" t="n">
-        <v>320</v>
+        <v>4.5</v>
       </c>
       <c r="P15" t="n">
-        <v>1600</v>
+        <v>45</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>BNB</t>
+          <t>UNI</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">

</xml_diff>